<commit_message>
Leads: 2026-10-28 05:00 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://groomsappliance.com/ac-installation/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>alana@groomsappliance.com</t>
@@ -614,6 +613,126 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Zion Home Roofing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>zionhomeroof.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.zionhomeroof.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>When David</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>davidh@zionhomeroof.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(513) 633-9084</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>residential roofing company Cincinnati OH</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Elevate Heating and Air</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>elevateairutah.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://elevateairutah.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Book Service</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>elevateairutah@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(435) 695-6348</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>heating and cooling company Ogden UT</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 05:07 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HVAC Company Mobile AL | Action Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>callaction.net</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.callaction.net/locations/mobile-al-hvac</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Action Heating</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>service@callaction.net</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(251) 272-5900</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Mobile AL</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>furnace repair Mobile AL</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 05:09 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Plumbing Pros Local</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>plumbingproslocal.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://plumbingproslocal.com/idaho/pocatello/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pros Local</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>service@plumbingproslocal.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>877-365-2933</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Pocatello ID</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>emergency plumber Pocatello ID</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:19 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Roofing Company in Huntsville, AL | Repair and Replacement</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>huntsvilleroofingco.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://huntsvilleroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Madison County</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>hello@huntsvilleroofingco.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(256) 583-9659</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>residential roofing company Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:28 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RISE Roofing &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>riseroofingandrestoration.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://riseroofingandrestoration.com/asheville/roof-repair</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Free Inspection</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@riseroofingandrestoration.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(704) 486-1348</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof repair company Asheville NC</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:34 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in West Palm Beach, FL | CLS Roofing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>clsroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.clsroofingllc.com/service-areas/west-palm-beach-fl</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Get Tips</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@clsroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(954) 743-5416</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:38 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1038,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ichiban Roofing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ichibanroofing.net</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://ichibanroofing.net/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Happy Customers</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@ichibanroofing.net</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(323) 295-4400</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofer Torrance CA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:42 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,62 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>R &amp; S Plumbing | Repairs and Replacements | Murfreesboro, TN</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>randsplumbingtn.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.randsplumbingtn.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ricky.england@comcast.net</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(615) 895-0867</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>plumber Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:44 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1119,7 +1119,6 @@
           <t>https://www.randsplumbingtn.com/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>ricky.england@comcast.net</t>
@@ -1149,6 +1148,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Roto-Rooter of Eastern Idaho</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rotorootereastidaho.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://rotorootereastidaho.com/clogged-drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Idaho Falls</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>wrotorooter@gmail.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(208) 523-4212</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>drain cleaning service Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:47 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1213,6 +1213,62 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>www.PoppyPlumbing.com</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>poppyplumbing.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://poppyplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>hello@poppyplumbing.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>86</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>plumbing company Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:49 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1244,7 +1244,6 @@
           <t>hello@poppyplumbing.com</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Los Angeles CA</t>
@@ -1264,6 +1263,62 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pennsylvania Connection</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>pennsylvaniaconnection.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://pennsylvaniaconnection.com/allentown/plumbers/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@pennsylvaniaconnection.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(484) 268-1364</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Allentown PA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>plumber Allentown PA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:55 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1289,7 +1289,6 @@
           <t>https://pennsylvaniaconnection.com/allentown/plumbers/</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@pennsylvaniaconnection.com</t>
@@ -1319,6 +1318,66 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OKC Water Heaters</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>okcwaterheaters.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://okcwaterheaters.com/services/water-heater-repair-oklahoma-city-ok</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Why Oklahoma</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@okcwaterheaters.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(405) 656-7895</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>94</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>water heater repair Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 15:59 UTC (cycle 33)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1383,6 +1383,114 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nelsonroofcontracting.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://nelsonroofcontracting.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>roofcontract@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>361-683-1733</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>78</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>roofing contractor Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Florida Roof Price</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>floridaroofprice.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://floridaroofprice.com/roofing-companies/pembroke-pines/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>hello@floridaroofprice.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>76</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>residential roofing company Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:01 UTC (cycle 34)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1404,7 +1404,6 @@
           <t>https://nelsonroofcontracting.com/</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>roofcontract@yahoo.com</t>
@@ -1460,13 +1459,11 @@
           <t>https://floridaroofprice.com/roofing-companies/pembroke-pines/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>hello@floridaroofprice.com</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Pembroke Pines FL</t>
@@ -1486,6 +1483,62 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HVAC Contractor in Brooklyn, NY | Cool Tech HVAC Corp</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>cooltechhvac.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.cooltechhvac.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>cooltech2@verizon.net</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(718) 668-2031</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>HVAC contractor Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:03 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1509,7 +1509,6 @@
           <t>https://www.cooltechhvac.com/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>cooltech2@verizon.net</t>
@@ -1539,6 +1538,62 @@
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Pride Roofing and Construction, LLC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>prideroofingandsolar.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.prideroofingandsolar.com/cheyenne</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@prideroofingandsolar.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(307) 277-4441</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>roofer Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:07 UTC (cycle 37)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1564,7 +1564,6 @@
           <t>https://www.prideroofingandsolar.com/cheyenne</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>info@prideroofingandsolar.com</t>
@@ -1594,6 +1593,66 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Davenport, IA - Midwest Roof &amp; Solar</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>midwestroofandsolar.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://midwestroofandsolar.com/iowa/davenport-ia/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Midwest Agriculture</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@midwestroofandsolar.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>651-383-1977</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>88</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roof replacement Davenport IA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:13 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1658,6 +1658,122 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Tech</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>waterheaterrepairtech.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://waterheaterrepairtech.com/michigan/troy/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Testimonials What</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>service@waterheaterrepairtech.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(877) 415-0636</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Troy MI</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>84</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>water heater repair Troy MI</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Runhome</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>runhome.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.runhome.com/locations/cities/troy-mi</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Michigan Short</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>hello@runhome.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Troy MI</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>76</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>water heater repair Troy MI</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:15 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1749,7 +1749,6 @@
           <t>hello@runhome.com</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Troy MI</t>
@@ -1769,6 +1768,174 @@
         </is>
       </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Roofing Of Athens</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>roofingofathens.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://roofingofathens.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>roofingofathens@gmail.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(706) 268-9998</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Athens GA</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>96</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>roofing contractor Athens GA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation and Replacement in Annapolis, MD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>annapolis-md.centralheatairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://annapolis-md.centralheatairconditioning.com/heat-pump-installation-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>contact@centralheatairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(833) 435-6630</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>heat pump installation Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ABF Roofing and Foam</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>abfroofinglubbock.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://abfroofinglubbock.com/our-work/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>robert@abfroofinglubbock.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(806) 863-3626</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Lubbock TX</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>90</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>residential roofing company Lubbock TX</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:17 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1794,7 +1794,6 @@
           <t>https://roofingofathens.com/</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>roofingofathens@gmail.com</t>
@@ -1850,7 +1849,6 @@
           <t>https://annapolis-md.centralheatairconditioning.com/heat-pump-installation-and-replacement/</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>contact@centralheatairconditioning.com</t>
@@ -1906,7 +1904,6 @@
           <t>https://abfroofinglubbock.com/our-work/residential-roofing/</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>robert@abfroofinglubbock.com</t>
@@ -1936,6 +1933,122 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Plumb Right | Expert Plumbing Services in Birmingham, AL</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>plumbrightfirst.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://plumbrightfirst.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>plumbright17@gmail.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(205) 202-2054</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>90</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>plumber Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Direct Line Plumbing Drain Gas &amp; Water LLC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>birminghamplumbingnearme.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://birminghamplumbingnearme.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Who Is</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>directlineal@gmail.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(205) 470-9566</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>plumber Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:19 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1959,7 +1959,6 @@
           <t>https://plumbrightfirst.com/</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>plumbright17@gmail.com</t>
@@ -2049,6 +2048,66 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mortelliti Contractors Inc</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>mortelliticontractors.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.mortelliticontractors.com/roof-replacement-in-stamford-ct/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>mortelliti@mortelliticontractors.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(914) 592-6860</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>90</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roof replacement Stamford CT</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:23 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2113,6 +2113,66 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Torrance, CA | 24/7 Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>expressplumbertorrance.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://expressplumbertorrance.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Rancho Palos</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>contact@expressplumbertorrance.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(310) 424-7510</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>emergency plumber Torrance CA</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:28 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2173,6 +2173,66 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Great White Mechanical Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>greatwhitemech.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://greatwhitemech.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Dave Owner</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>greatwhitemech@outlook.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(941) 342-6595</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>86</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:43 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2233,6 +2233,66 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1 Honest Plumber</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1honestplumber.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://1honestplumber.com/emergency-services/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ed.1honestplumber@gmail.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>650-422-4736</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>emergency plumber Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:49 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2293,6 +2293,122 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Roofing, Replacement Windows, Baths &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>rooftopdesigns.net</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://rooftopdesigns.net/locations/maryland/rockville-md/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>yanni@rooftopdesigns.net</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>855-662-7388</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Rockville MD</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>100</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>residential roofing company Rockville MD</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Roof Repair &amp; Replacement Danbury | EDM Construction</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>edmconstructionct.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.edmconstructionct.com/services/roofing-replacements-repairs</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Speak With</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>edmconstruction64@gmail.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(203) 567-7490</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Danbury CT</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>90</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>roof replacement Danbury CT</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:51 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2314,7 +2314,6 @@
           <t>https://rooftopdesigns.net/locations/maryland/rockville-md/</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>yanni@rooftopdesigns.net</t>
@@ -2404,6 +2403,66 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>leak detection mckinney</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>leakdetectionmckinney.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.leakdetectionmckinney.com/services/sewer-line-leak-repair.html</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Mark Thompson</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>leakdetectionmckinney@gmail.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(469) 837-2954</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>sewer repair McKinney TX</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:53 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2468,6 +2468,126 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Element Heating Cooling and Refrigeration</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>elementhvacr.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://elementhvacr.com/parma-oh/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Commercial Expertise</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>mike.pontious@elementhvacr.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>1216815589</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Parma OH</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>heating and cooling company Parma OH</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Elite Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>elitemetalroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://elitemetalroofingllc.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Portland Request</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>robert@elitemetalroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>360-487-9090</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 16:57 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2588,6 +2588,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wolf Roofing</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>wolfroofing.net</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://wolfroofing.net/service-areas/ankeny/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Another Wolf</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>admin@wolfconstruction.net</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(515) 225-8866</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>100</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>roofing contractor Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 17:10 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2648,6 +2648,62 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Heating Repair, Tune-Ups, and Installation in Harrisburg, PA</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>countrysidefuel.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.countrysidefuel.com/service-areas/heating-services-harrisburg</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@countrysidefuel.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(610) 314-0294</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>furnace repair Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 20:53 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2669,7 +2669,6 @@
           <t>https://www.countrysidefuel.com/service-areas/heating-services-harrisburg</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>info@countrysidefuel.com</t>
@@ -2699,6 +2698,66 @@
         </is>
       </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Furnace Repair in Kansas City | Expert Heating Service | Luna Heating and Coolin</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>lunaheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.lunaheatingcooling.com/heating/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Read More</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>support@lunaheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(913) 283-1018</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>100</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>furnace repair Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-28 20:55 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2763,6 +2763,66 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bella Construction &amp; Development Inc. - Pittsburgh Residential Roofing &amp; Siding </t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>mybellaroof.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://mybellaroof.com/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Western Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>info@mybellaroof.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(724) 515-5163</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>100</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-28 21:07 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-28.xlsx
+++ b/output/leads_2026-10-28.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2823,6 +2823,122 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AC Repair Erie PA | Same-Day AC Repair in Erie &amp; the Erie region</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>hvacerie.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://hvacerie.com/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Policy Terms</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>info@hvacerie.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(814) 447-4494</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Erie PA</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>AC installation Erie PA</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Dr. Cool, Inc.</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>drcooldrheat.net</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://drcooldrheat.net/residential/air-conditioning/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>noreply@drcooldrheat.net</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>253.863.5665</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Tacoma WA</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>90</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>air conditioning repair Tacoma WA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>